<commit_message>
Add educational quality analysis, statewide benchmarks, TOC link fixes, facility suitability, and final public review
Incorporates state assessment data for all RSU 5 schools, school consolidation research, MSS outdoor space/Chapter 124 compliance analysis, statewide per-pupil expenditure benchmarks, and Finance Committee document archive. Final review pass ensures consistency, sanitized workbooks, and corrected TOC linking across both public documents.
</commit_message>
<xml_diff>
--- a/RSU5 Overview FY17-FY29.xlsx
+++ b/RSU5 Overview FY17-FY29.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enrollment" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Staffing FTE" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Article Growth" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C-SchoolBudgets" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,8 +20,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="6">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="+#,##0;-#,##0"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,6 +54,9 @@
       <b val="1"/>
       <color rgb="00C00000"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="6">
@@ -98,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -124,6 +131,10 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1635,4 +1646,924 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="23" t="inlineStr">
+        <is>
+          <t>CALC: School-Level Budget Comparison (FY22-FY27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>All values are adopted budgets from I-BudgetData in each fiscal year workbook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Direct school costs = Articles 1 + 2 + 4 + 5 + 7 + 9 allocated to each building.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Enrollment from Superintendent Handbooks (Oct 1 headcounts). See I-BudgetData in FY22-FY27 workbooks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Growth rates: CAGR = (End/Start)^(1/years) - 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>1. DIRECT SCHOOL BUDGETS (Adopted, Articles 1+2+4+5+7+9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>School</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>FY22</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>FY23</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="E8" s="23" t="inlineStr">
+        <is>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="inlineStr">
+        <is>
+          <t>FY26</t>
+        </is>
+      </c>
+      <c r="G8" s="23" t="inlineStr">
+        <is>
+          <t>FY27</t>
+        </is>
+      </c>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>$ Change</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>% Change</t>
+        </is>
+      </c>
+      <c r="J8" s="23" t="inlineStr">
+        <is>
+          <t>CAGR</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DCS</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="n">
+        <v>5509152</v>
+      </c>
+      <c r="C9" s="24" t="n">
+        <v>5970223</v>
+      </c>
+      <c r="D9" s="24" t="n">
+        <v>6349743</v>
+      </c>
+      <c r="E9" s="24" t="n">
+        <v>6903159</v>
+      </c>
+      <c r="F9" s="24" t="n">
+        <v>7444449</v>
+      </c>
+      <c r="G9" s="24" t="n">
+        <v>8035575</v>
+      </c>
+      <c r="H9" s="25" t="n">
+        <v>2526423</v>
+      </c>
+      <c r="I9" s="26" t="n">
+        <v>0.4585865483471867</v>
+      </c>
+      <c r="J9" s="26" t="n">
+        <v>0.07841629331104549</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MSS</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="n">
+        <v>3478156</v>
+      </c>
+      <c r="C10" s="24" t="n">
+        <v>3806987</v>
+      </c>
+      <c r="D10" s="24" t="n">
+        <v>4160223</v>
+      </c>
+      <c r="E10" s="24" t="n">
+        <v>4480324</v>
+      </c>
+      <c r="F10" s="24" t="n">
+        <v>4659054</v>
+      </c>
+      <c r="G10" s="24" t="n">
+        <v>4942823</v>
+      </c>
+      <c r="H10" s="25" t="n">
+        <v>1464667</v>
+      </c>
+      <c r="I10" s="26" t="n">
+        <v>0.4211044587994328</v>
+      </c>
+      <c r="J10" s="26" t="n">
+        <v>0.07281589735163063</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PES</t>
+        </is>
+      </c>
+      <c r="B11" s="24" t="n">
+        <v>1645284</v>
+      </c>
+      <c r="C11" s="24" t="n">
+        <v>1868327</v>
+      </c>
+      <c r="D11" s="24" t="n">
+        <v>1859665</v>
+      </c>
+      <c r="E11" s="24" t="n">
+        <v>1992101</v>
+      </c>
+      <c r="F11" s="24" t="n">
+        <v>2158007</v>
+      </c>
+      <c r="G11" s="24" t="n">
+        <v>2270105</v>
+      </c>
+      <c r="H11" s="25" t="n">
+        <v>624821</v>
+      </c>
+      <c r="I11" s="26" t="n">
+        <v>0.3797648308741834</v>
+      </c>
+      <c r="J11" s="26" t="n">
+        <v>0.06650037916020968</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>MLS</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="n">
+        <v>3197486</v>
+      </c>
+      <c r="C12" s="24" t="n">
+        <v>3466532</v>
+      </c>
+      <c r="D12" s="24" t="n">
+        <v>3545024</v>
+      </c>
+      <c r="E12" s="24" t="n">
+        <v>4053005</v>
+      </c>
+      <c r="F12" s="24" t="n">
+        <v>4408771</v>
+      </c>
+      <c r="G12" s="24" t="n">
+        <v>4568270</v>
+      </c>
+      <c r="H12" s="25" t="n">
+        <v>1370784</v>
+      </c>
+      <c r="I12" s="26" t="n">
+        <v>0.4287068027819356</v>
+      </c>
+      <c r="J12" s="26" t="n">
+        <v>0.07396127676097541</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>FMS</t>
+        </is>
+      </c>
+      <c r="B13" s="24" t="n">
+        <v>4635126</v>
+      </c>
+      <c r="C13" s="24" t="n">
+        <v>4937218</v>
+      </c>
+      <c r="D13" s="24" t="n">
+        <v>5456378</v>
+      </c>
+      <c r="E13" s="24" t="n">
+        <v>5678540</v>
+      </c>
+      <c r="F13" s="24" t="n">
+        <v>5964288</v>
+      </c>
+      <c r="G13" s="24" t="n">
+        <v>6136815</v>
+      </c>
+      <c r="H13" s="25" t="n">
+        <v>1501689</v>
+      </c>
+      <c r="I13" s="26" t="n">
+        <v>0.3239801895353007</v>
+      </c>
+      <c r="J13" s="26" t="n">
+        <v>0.05773359267439782</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>FHS</t>
+        </is>
+      </c>
+      <c r="B14" s="24" t="n">
+        <v>8837419</v>
+      </c>
+      <c r="C14" s="24" t="n">
+        <v>8904609</v>
+      </c>
+      <c r="D14" s="24" t="n">
+        <v>8865428</v>
+      </c>
+      <c r="E14" s="24" t="n">
+        <v>9929358</v>
+      </c>
+      <c r="F14" s="24" t="n">
+        <v>10029663</v>
+      </c>
+      <c r="G14" s="24" t="n">
+        <v>10481438</v>
+      </c>
+      <c r="H14" s="25" t="n">
+        <v>1644019</v>
+      </c>
+      <c r="I14" s="26" t="n">
+        <v>0.1860293146675518</v>
+      </c>
+      <c r="J14" s="26" t="n">
+        <v>0.03471104431923888</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>RSU Total</t>
+        </is>
+      </c>
+      <c r="B15" s="24" t="n">
+        <v>35714863</v>
+      </c>
+      <c r="C15" s="24" t="n">
+        <v>37223151</v>
+      </c>
+      <c r="D15" s="24" t="n">
+        <v>39080569</v>
+      </c>
+      <c r="E15" s="24" t="n">
+        <v>41612460</v>
+      </c>
+      <c r="F15" s="24" t="n">
+        <v>44455929</v>
+      </c>
+      <c r="G15" s="24" t="n">
+        <v>47357441</v>
+      </c>
+      <c r="H15" s="25" t="n">
+        <v>11642578</v>
+      </c>
+      <c r="I15" s="26" t="n">
+        <v>0.3259869147475101</v>
+      </c>
+      <c r="J15" s="26" t="n">
+        <v>0.05805403477708992</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t>2. ENROLLMENT (Oct 1 headcounts from Superintendent Handbooks)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="23" t="inlineStr">
+        <is>
+          <t>School</t>
+        </is>
+      </c>
+      <c r="B18" s="23" t="inlineStr">
+        <is>
+          <t>Oct 2021</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>Oct 2022</t>
+        </is>
+      </c>
+      <c r="D18" s="23" t="inlineStr">
+        <is>
+          <t>Oct 2023</t>
+        </is>
+      </c>
+      <c r="E18" s="23" t="inlineStr">
+        <is>
+          <t>Oct 2024</t>
+        </is>
+      </c>
+      <c r="F18" s="23" t="inlineStr">
+        <is>
+          <t>Oct 2025</t>
+        </is>
+      </c>
+      <c r="G18" s="23" t="inlineStr">
+        <is>
+          <t>Oct 2026P</t>
+        </is>
+      </c>
+      <c r="H18" s="23" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="I18" s="23" t="inlineStr">
+        <is>
+          <t>% Change</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>DCS</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>455</v>
+      </c>
+      <c r="C19" t="n">
+        <v>463</v>
+      </c>
+      <c r="D19" t="n">
+        <v>473</v>
+      </c>
+      <c r="E19" t="n">
+        <v>466</v>
+      </c>
+      <c r="F19" t="n">
+        <v>453</v>
+      </c>
+      <c r="G19" t="n">
+        <v>467</v>
+      </c>
+      <c r="H19" t="n">
+        <v>12</v>
+      </c>
+      <c r="I19" s="26" t="n">
+        <v>0.02637362637362628</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>MSS</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>301</v>
+      </c>
+      <c r="C20" t="n">
+        <v>327</v>
+      </c>
+      <c r="D20" t="n">
+        <v>316</v>
+      </c>
+      <c r="E20" t="n">
+        <v>288</v>
+      </c>
+      <c r="F20" t="n">
+        <v>275</v>
+      </c>
+      <c r="G20" t="n">
+        <v>274</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-27</v>
+      </c>
+      <c r="I20" s="26" t="n">
+        <v>-0.0897009966777409</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>PES</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>108</v>
+      </c>
+      <c r="C21" t="n">
+        <v>96</v>
+      </c>
+      <c r="D21" t="n">
+        <v>89</v>
+      </c>
+      <c r="E21" t="n">
+        <v>97</v>
+      </c>
+      <c r="F21" t="n">
+        <v>98</v>
+      </c>
+      <c r="G21" t="n">
+        <v>105</v>
+      </c>
+      <c r="H21" t="n">
+        <v>-3</v>
+      </c>
+      <c r="I21" s="26" t="n">
+        <v>-0.02777777777777779</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>MLS</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>235</v>
+      </c>
+      <c r="C22" t="n">
+        <v>254</v>
+      </c>
+      <c r="D22" t="n">
+        <v>281</v>
+      </c>
+      <c r="E22" t="n">
+        <v>266</v>
+      </c>
+      <c r="F22" t="n">
+        <v>282</v>
+      </c>
+      <c r="G22" t="n">
+        <v>264</v>
+      </c>
+      <c r="H22" t="n">
+        <v>29</v>
+      </c>
+      <c r="I22" s="26" t="n">
+        <v>0.123404255319149</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>FMS</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>296</v>
+      </c>
+      <c r="C23" t="n">
+        <v>307</v>
+      </c>
+      <c r="D23" t="n">
+        <v>293</v>
+      </c>
+      <c r="E23" t="n">
+        <v>288</v>
+      </c>
+      <c r="F23" t="n">
+        <v>286</v>
+      </c>
+      <c r="G23" t="n">
+        <v>306</v>
+      </c>
+      <c r="H23" t="n">
+        <v>10</v>
+      </c>
+      <c r="I23" s="26" t="n">
+        <v>0.03378378378378377</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>FHS</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>595</v>
+      </c>
+      <c r="C24" t="n">
+        <v>619</v>
+      </c>
+      <c r="D24" t="n">
+        <v>632</v>
+      </c>
+      <c r="E24" t="n">
+        <v>592</v>
+      </c>
+      <c r="F24" t="n">
+        <v>577</v>
+      </c>
+      <c r="G24" t="n">
+        <v>554</v>
+      </c>
+      <c r="H24" t="n">
+        <v>-41</v>
+      </c>
+      <c r="I24" s="26" t="n">
+        <v>-0.06890756302521006</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1990</v>
+      </c>
+      <c r="C25" t="n">
+        <v>2066</v>
+      </c>
+      <c r="D25" t="n">
+        <v>2084</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1997</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1971</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1970</v>
+      </c>
+      <c r="H25" t="n">
+        <v>-20</v>
+      </c>
+      <c r="I25" s="26" t="n">
+        <v>-0.01005025125628145</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="23" t="inlineStr">
+        <is>
+          <t>3. PER-STUDENT COST (Adopted Budget / Oct 1 Enrollment)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="23" t="inlineStr">
+        <is>
+          <t>School</t>
+        </is>
+      </c>
+      <c r="B28" s="23" t="inlineStr">
+        <is>
+          <t>FY22</t>
+        </is>
+      </c>
+      <c r="C28" s="23" t="inlineStr">
+        <is>
+          <t>FY23</t>
+        </is>
+      </c>
+      <c r="D28" s="23" t="inlineStr">
+        <is>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="E28" s="23" t="inlineStr">
+        <is>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="F28" s="23" t="inlineStr">
+        <is>
+          <t>FY26</t>
+        </is>
+      </c>
+      <c r="G28" s="23" t="inlineStr">
+        <is>
+          <t>FY27</t>
+        </is>
+      </c>
+      <c r="H28" s="23" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="I28" s="23" t="inlineStr">
+        <is>
+          <t>% Change</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>DCS</t>
+        </is>
+      </c>
+      <c r="B29" s="24" t="n">
+        <v>12108</v>
+      </c>
+      <c r="C29" s="24" t="n">
+        <v>12895</v>
+      </c>
+      <c r="D29" s="24" t="n">
+        <v>13424</v>
+      </c>
+      <c r="E29" s="24" t="n">
+        <v>14814</v>
+      </c>
+      <c r="F29" s="24" t="n">
+        <v>16434</v>
+      </c>
+      <c r="G29" s="24" t="n">
+        <v>17207</v>
+      </c>
+      <c r="H29" s="25" t="n">
+        <v>5099</v>
+      </c>
+      <c r="I29" s="26" t="n">
+        <v>0.4211068083468308</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>MSS</t>
+        </is>
+      </c>
+      <c r="B30" s="24" t="n">
+        <v>11555</v>
+      </c>
+      <c r="C30" s="24" t="n">
+        <v>11642</v>
+      </c>
+      <c r="D30" s="24" t="n">
+        <v>13165</v>
+      </c>
+      <c r="E30" s="24" t="n">
+        <v>15557</v>
+      </c>
+      <c r="F30" s="24" t="n">
+        <v>16942</v>
+      </c>
+      <c r="G30" s="24" t="n">
+        <v>18040</v>
+      </c>
+      <c r="H30" s="25" t="n">
+        <v>6484</v>
+      </c>
+      <c r="I30" s="26" t="n">
+        <v>0.5611402996300339</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>PES</t>
+        </is>
+      </c>
+      <c r="B31" s="24" t="n">
+        <v>15234</v>
+      </c>
+      <c r="C31" s="24" t="n">
+        <v>19462</v>
+      </c>
+      <c r="D31" s="24" t="n">
+        <v>20895</v>
+      </c>
+      <c r="E31" s="24" t="n">
+        <v>20537</v>
+      </c>
+      <c r="F31" s="24" t="n">
+        <v>22020</v>
+      </c>
+      <c r="G31" s="24" t="n">
+        <v>21620</v>
+      </c>
+      <c r="H31" s="25" t="n">
+        <v>6386</v>
+      </c>
+      <c r="I31" s="26" t="n">
+        <v>0.4191866831848743</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>MLS</t>
+        </is>
+      </c>
+      <c r="B32" s="24" t="n">
+        <v>13606</v>
+      </c>
+      <c r="C32" s="24" t="n">
+        <v>13648</v>
+      </c>
+      <c r="D32" s="24" t="n">
+        <v>12616</v>
+      </c>
+      <c r="E32" s="24" t="n">
+        <v>15237</v>
+      </c>
+      <c r="F32" s="24" t="n">
+        <v>15634</v>
+      </c>
+      <c r="G32" s="24" t="n">
+        <v>17304</v>
+      </c>
+      <c r="H32" s="25" t="n">
+        <v>3698</v>
+      </c>
+      <c r="I32" s="26" t="n">
+        <v>0.2717655252036169</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>FMS</t>
+        </is>
+      </c>
+      <c r="B33" s="24" t="n">
+        <v>15659</v>
+      </c>
+      <c r="C33" s="24" t="n">
+        <v>16082</v>
+      </c>
+      <c r="D33" s="24" t="n">
+        <v>18622</v>
+      </c>
+      <c r="E33" s="24" t="n">
+        <v>19717</v>
+      </c>
+      <c r="F33" s="24" t="n">
+        <v>20854</v>
+      </c>
+      <c r="G33" s="24" t="n">
+        <v>20055</v>
+      </c>
+      <c r="H33" s="25" t="n">
+        <v>4396</v>
+      </c>
+      <c r="I33" s="26" t="n">
+        <v>0.2807128630798987</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>FHS</t>
+        </is>
+      </c>
+      <c r="B34" s="24" t="n">
+        <v>14853</v>
+      </c>
+      <c r="C34" s="24" t="n">
+        <v>14385</v>
+      </c>
+      <c r="D34" s="24" t="n">
+        <v>14028</v>
+      </c>
+      <c r="E34" s="24" t="n">
+        <v>16773</v>
+      </c>
+      <c r="F34" s="24" t="n">
+        <v>17382</v>
+      </c>
+      <c r="G34" s="24" t="n">
+        <v>18920</v>
+      </c>
+      <c r="H34" s="25" t="n">
+        <v>4067</v>
+      </c>
+      <c r="I34" s="26" t="n">
+        <v>0.273804047341504</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="23" t="inlineStr">
+        <is>
+          <t>4. METHODOLOGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Budget source: I-BudgetData sheet in each FY workbook (FY22-FY26), I-Budget in FY27.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Direct costs = sum of Articles 1, 2, 4, 5, 7, 9 for each cost center (school).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>System-wide articles (3, 6, 8, 10, 11) are NOT included; they are shared across all schools.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Enrollment source: Oct 1 headcounts from Superintendent Handbooks, matched to fiscal year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>FY22 uses Oct 2021 count; FY27 uses Oct 2026 projected. Enrollment is for the school year starting that fiscal year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>CAGR = Compound Annual Growth Rate = (FY27/FY22)^(1/5) - 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Per-student cost = Direct budget / Oct 1 enrollment for the corresponding year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Referenced in: Omnibus Sections 3.3, 3.4, Executive Summary.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>